<commit_message>
Updated Steam Achivement Data to use one consistent source
</commit_message>
<xml_diff>
--- a/Steam Achievements.xlsx
+++ b/Steam Achievements.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="79">
   <si>
     <t>Game</t>
   </si>
@@ -31,265 +31,223 @@
     <t>Image_Link</t>
   </si>
   <si>
-    <t>Cuphead</t>
-  </si>
-  <si>
-    <t>Taking Names</t>
-  </si>
-  <si>
-    <t>Parry Persistance</t>
-  </si>
-  <si>
-    <t>Parry Performance</t>
-  </si>
-  <si>
-    <t>Cutting Corners</t>
-  </si>
-  <si>
-    <t>A Walk in the Park</t>
-  </si>
-  <si>
-    <t>Perfect Run</t>
-  </si>
-  <si>
-    <t>Ceramic Strike</t>
-  </si>
-  <si>
-    <t>A Day at the Fair</t>
-  </si>
-  <si>
-    <t>Porcelain Power</t>
-  </si>
-  <si>
-    <t>Magician Lord</t>
-  </si>
-  <si>
-    <t>A Trip Downtown</t>
-  </si>
-  <si>
-    <t>Bouncing Ball</t>
-  </si>
-  <si>
-    <t>Casino Night</t>
-  </si>
-  <si>
-    <t>Souls Saved</t>
-  </si>
-  <si>
-    <t>Swing You Sinner</t>
-  </si>
-  <si>
-    <t>Alive and Kicking</t>
-  </si>
-  <si>
-    <t>Coffers Full</t>
-  </si>
-  <si>
-    <t>The Latest Sensation</t>
-  </si>
-  <si>
-    <t>Selling Out</t>
-  </si>
-  <si>
-    <t>Butter-and-Egg Man</t>
-  </si>
-  <si>
-    <t>Sheriff</t>
-  </si>
-  <si>
-    <t>King</t>
-  </si>
-  <si>
-    <t>A Vacation in the Wilds</t>
-  </si>
-  <si>
-    <t>Put On a Show</t>
-  </si>
-  <si>
-    <t>Compliments to the Chef</t>
-  </si>
-  <si>
-    <t>Checkmate</t>
-  </si>
-  <si>
-    <t>High Roller</t>
-  </si>
-  <si>
-    <t>Rolling Sixes</t>
-  </si>
-  <si>
-    <t>A Horrible Night To Have a Curse</t>
-  </si>
-  <si>
-    <t>Boss</t>
-  </si>
-  <si>
-    <t>The Golden Touch</t>
-  </si>
-  <si>
-    <t>Decadent</t>
-  </si>
-  <si>
-    <t>Mayor</t>
-  </si>
-  <si>
-    <t>Pacifist</t>
-  </si>
-  <si>
-    <t>Hearty</t>
-  </si>
-  <si>
-    <t>Paladin</t>
-  </si>
-  <si>
-    <t>Bravo Zulu P-26</t>
-  </si>
-  <si>
-    <t>Beat The Devil At His Own Game</t>
-  </si>
-  <si>
-    <t>A King's Admiration</t>
-  </si>
-  <si>
-    <t>Ranger</t>
-  </si>
-  <si>
-    <t>The High Hat</t>
-  </si>
-  <si>
-    <t>Cooked to Perfection</t>
-  </si>
-  <si>
-    <t>Defeat a boss</t>
-  </si>
-  <si>
-    <t>Complete 20 parries</t>
-  </si>
-  <si>
-    <t>Complete 100 parries</t>
-  </si>
-  <si>
-    <t>Find a shortcut</t>
-  </si>
-  <si>
-    <t>Defeat every boss in Inkwell Isle I</t>
-  </si>
-  <si>
-    <t>Complete a level without getting hit</t>
-  </si>
-  <si>
-    <t>Defeat a boss with an Extra Special move</t>
-  </si>
-  <si>
-    <t>Defeat every boss in Inkwell Isle II</t>
-  </si>
-  <si>
-    <t>Defeat a boss with a Super Art</t>
-  </si>
-  <si>
-    <t>Obtain all Super Arts</t>
-  </si>
-  <si>
-    <t>Defeat every boss in Inkwell Isle III</t>
-  </si>
-  <si>
-    <t>Parry five times before hitting the ground</t>
-  </si>
-  <si>
-    <t>Complete the Casino</t>
-  </si>
-  <si>
-    <t>Complete the game on Normal</t>
-  </si>
-  <si>
-    <t>Defeat the Devil</t>
-  </si>
-  <si>
-    <t>Defeat a boss with Ms. Chalice</t>
-  </si>
-  <si>
-    <t>Get every coin in all of the levels</t>
-  </si>
-  <si>
-    <t>Defeat a boss with one of Porkrind's new weapons</t>
-  </si>
-  <si>
-    <t>Give in to the Devil</t>
-  </si>
-  <si>
-    <t>Buy everything in Porkrind's Shop</t>
-  </si>
-  <si>
-    <t>Obtain an A-Rank or higher on all bosses in Inkwell Isle I</t>
-  </si>
-  <si>
-    <t>Obtain an A-Rank or higher on all bosses in Inkwell Hell</t>
-  </si>
-  <si>
-    <t>Defeat every boss in Inkwell Isle IV</t>
-  </si>
-  <si>
-    <t>Get an S-Rank</t>
-  </si>
-  <si>
-    <t>Complete your quest on Inkwell Isle IV</t>
-  </si>
-  <si>
-    <t>Defeat all of the King of Games' Champions</t>
-  </si>
-  <si>
-    <t>Get every coin in the game</t>
-  </si>
-  <si>
-    <t>Defeat King Dice without taking a hit</t>
-  </si>
-  <si>
-    <t>Survive the nightmare</t>
-  </si>
-  <si>
-    <t>Obtain an A-Rank or higher on all bosses in Inkwell Isle II</t>
-  </si>
-  <si>
-    <t>Defeat a boss with one of Ms. Chalice's Super Arts</t>
-  </si>
-  <si>
-    <t>Defeat 10 bosses with Ms. Chalice</t>
-  </si>
-  <si>
-    <t>Obtain an A-Rank or higher on all bosses in Inkwell Isle III</t>
-  </si>
-  <si>
-    <t>Complete all levels without killing an enemy</t>
-  </si>
-  <si>
-    <t>Have 9HP at one time</t>
-  </si>
-  <si>
-    <t>Obtain great power</t>
-  </si>
-  <si>
-    <t>Defeat a boss using only the mini-plane bullets</t>
-  </si>
-  <si>
-    <t>Complete the game on Expert</t>
-  </si>
-  <si>
-    <t>Defeat the King's Gauntlet</t>
-  </si>
-  <si>
-    <t>Obtain an A-Rank or Higher on all bosses in Inkwell Isle IV</t>
-  </si>
-  <si>
-    <t>Defeat a boss on Inkwell Isle IV without killing any of its minions</t>
-  </si>
-  <si>
-    <t>Get an S-Rank on a stage of Inkwell Isle IV</t>
-  </si>
-  <si>
-    <t>https://shared.fastly.steamstatic.com/community_assets/images/apps/268910/7f66cff96c3f74ce806ed5d311a52a11bbbce43e.jpg</t>
-  </si>
-  <si>
-    <t>https://shared.fastly.steamstatic.com/community_assets/images/apps/268910/f768e3f225fe867e1eea454991b8ce290ce5b641.jpg</t>
+    <t>Nine Sols</t>
+  </si>
+  <si>
+    <t>My Revenge Starts Here</t>
+  </si>
+  <si>
+    <t>I'm Coming for You, Old Friend</t>
+  </si>
+  <si>
+    <t>Reap What You Sow</t>
+  </si>
+  <si>
+    <t>You Should Respect Your Elders</t>
+  </si>
+  <si>
+    <t>Jail Break</t>
+  </si>
+  <si>
+    <t>No Pain, No Gain</t>
+  </si>
+  <si>
+    <t>Wake Up From My Sin</t>
+  </si>
+  <si>
+    <t>The Cavalry's Here</t>
+  </si>
+  <si>
+    <t>Do Re Mi So La</t>
+  </si>
+  <si>
+    <t>Come, Sweet Death</t>
+  </si>
+  <si>
+    <t>We Have Each Other</t>
+  </si>
+  <si>
+    <t>Gimme Gimme</t>
+  </si>
+  <si>
+    <t>Across Time and Space</t>
+  </si>
+  <si>
+    <t>Magical Bean</t>
+  </si>
+  <si>
+    <t>Fight Dirty</t>
+  </si>
+  <si>
+    <t>You Bastard...</t>
+  </si>
+  <si>
+    <t>Stonks!</t>
+  </si>
+  <si>
+    <t>Evolution</t>
+  </si>
+  <si>
+    <t>Learned From the Best</t>
+  </si>
+  <si>
+    <t>One Man Army</t>
+  </si>
+  <si>
+    <t>I'm Yi, I Have a Drinking Problem</t>
+  </si>
+  <si>
+    <t>Blessed Messages</t>
+  </si>
+  <si>
+    <t>Passing on the Torch</t>
+  </si>
+  <si>
+    <t>Fight Through Hardship</t>
+  </si>
+  <si>
+    <t>The Warrior Within</t>
+  </si>
+  <si>
+    <t>Well Prepared</t>
+  </si>
+  <si>
+    <t>Home Sweet Home</t>
+  </si>
+  <si>
+    <t>Found You</t>
+  </si>
+  <si>
+    <t>Shooting Star</t>
+  </si>
+  <si>
+    <t>My Most Trusted Friend</t>
+  </si>
+  <si>
+    <t>Rest for the Wicked</t>
+  </si>
+  <si>
+    <t>What Have You Done?!</t>
+  </si>
+  <si>
+    <t>Repurposed</t>
+  </si>
+  <si>
+    <t>Treasure Hunter</t>
+  </si>
+  <si>
+    <t>Robo Fight!</t>
+  </si>
+  <si>
+    <t>Defeat Baichang.</t>
+  </si>
+  <si>
+    <t>Defeat Yingzhao.</t>
+  </si>
+  <si>
+    <t>Defeat Goumang.</t>
+  </si>
+  <si>
+    <t>Defeat Yanlao.</t>
+  </si>
+  <si>
+    <t>Successfully escape from prison.</t>
+  </si>
+  <si>
+    <t>Defeat Jiequan.</t>
+  </si>
+  <si>
+    <t>Defeat Lady Ethereal.</t>
+  </si>
+  <si>
+    <t>Rescue the people of the Peach Blossom Village.</t>
+  </si>
+  <si>
+    <t>Unravel the mystery of the Daybreak Tower's music sheet.</t>
+  </si>
+  <si>
+    <t>Defeat Ji.</t>
+  </si>
+  <si>
+    <t>Defeat Fuxi and Nuwa.</t>
+  </si>
+  <si>
+    <t>Establish a deep relationship with Shuanshuan.</t>
+  </si>
+  <si>
+    <t>Bid farewell to Lear.</t>
+  </si>
+  <si>
+    <t>Help Shuanshuan unlock the true potential of agriculture.</t>
+  </si>
+  <si>
+    <t>Use the Gene Eradicator to fight Jiequan.</t>
+  </si>
+  <si>
+    <t>Obtain map data from Shanhai 9000 by force.</t>
+  </si>
+  <si>
+    <t>Recycle Shuanshuan's coin.</t>
+  </si>
+  <si>
+    <t>Discover a tremendous secret.</t>
+  </si>
+  <si>
+    <t>Defeat Eigong.</t>
+  </si>
+  <si>
+    <t>Defeat every optional miniboss.</t>
+  </si>
+  <si>
+    <t>Drink all the wine brewed by Shennong.</t>
+  </si>
+  <si>
+    <t>Discover the message board for blessings upon the Departure of New Kunlun's Voyage.</t>
+  </si>
+  <si>
+    <t>Help Shennong become the leader of Peach Blossom Village.</t>
+  </si>
+  <si>
+    <t>Finish Nine Sols on Standard Mode.</t>
+  </si>
+  <si>
+    <t>Master all skills in the skill tree.</t>
+  </si>
+  <si>
+    <t>Collect every Jade.</t>
+  </si>
+  <si>
+    <t>Return to the home world of Solarian.</t>
+  </si>
+  <si>
+    <t>Help Shanhai 9000 find Chien.</t>
+  </si>
+  <si>
+    <t>Witness the end of New Kunlun.</t>
+  </si>
+  <si>
+    <t>Max out the ammo capacity of the Azure Bow and obtain Cloud Piercer X, Thunder Buster X, and Shadow Hunter X.</t>
+  </si>
+  <si>
+    <t>Help Chiyou bring peace to Xingtian.</t>
+  </si>
+  <si>
+    <t>Break the clay pot made by Shuanshuan</t>
+  </si>
+  <si>
+    <t>Use the Fortune teller machine crafted by Shuanshuan.</t>
+  </si>
+  <si>
+    <t>Find all resources and information marked by Shanhai 9000.</t>
+  </si>
+  <si>
+    <t>Defeat Tianshou while driving a robot.</t>
+  </si>
+  <si>
+    <t>https://shared.fastly.steamstatic.com/community_assets/images/apps/1809540/ca9a9a14d38e544a2edb077827f195baae480558.jpg</t>
+  </si>
+  <si>
+    <t>https://shared.fastly.steamstatic.com/community_assets/images/apps/1809540/034d35829e92d3ebd7743eff871e3111999aa2f9.jpg</t>
   </si>
   <si>
     <t>data:,</t>
@@ -663,7 +621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F43"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -694,13 +652,13 @@
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="E2">
-        <v>0.7659999999999999</v>
+        <v>0.8340000000000001</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>90</v>
+        <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -714,13 +672,13 @@
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="E3">
-        <v>0.7509999999999999</v>
+        <v>0.588</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -734,13 +692,13 @@
         <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E4">
-        <v>0.59</v>
+        <v>0.476</v>
       </c>
       <c r="F4" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -754,13 +712,13 @@
         <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="E5">
-        <v>0.545</v>
+        <v>0.418</v>
       </c>
       <c r="F5" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -774,13 +732,13 @@
         <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="E6">
-        <v>0.5329999999999999</v>
+        <v>0.401</v>
       </c>
       <c r="F6" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -794,13 +752,13 @@
         <v>11</v>
       </c>
       <c r="D7" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="E7">
-        <v>0.457</v>
+        <v>0.373</v>
       </c>
       <c r="F7" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -814,13 +772,13 @@
         <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E8">
-        <v>0.41</v>
+        <v>0.359</v>
       </c>
       <c r="F8" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -834,13 +792,13 @@
         <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="E9">
-        <v>0.313</v>
+        <v>0.355</v>
       </c>
       <c r="F9" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -854,13 +812,13 @@
         <v>14</v>
       </c>
       <c r="D10" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E10">
-        <v>0.282</v>
+        <v>0.345</v>
       </c>
       <c r="F10" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -874,13 +832,13 @@
         <v>15</v>
       </c>
       <c r="D11" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="E11">
-        <v>0.241</v>
+        <v>0.332</v>
       </c>
       <c r="F11" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -894,13 +852,13 @@
         <v>16</v>
       </c>
       <c r="D12" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="E12">
-        <v>0.219</v>
+        <v>0.326</v>
       </c>
       <c r="F12" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -914,13 +872,13 @@
         <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E13">
-        <v>0.215</v>
+        <v>0.323</v>
       </c>
       <c r="F13" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -934,13 +892,13 @@
         <v>18</v>
       </c>
       <c r="D14" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="E14">
-        <v>0.184</v>
+        <v>0.3</v>
       </c>
       <c r="F14" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -954,13 +912,13 @@
         <v>19</v>
       </c>
       <c r="D15" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E15">
-        <v>0.174</v>
+        <v>0.292</v>
       </c>
       <c r="F15" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -974,13 +932,13 @@
         <v>20</v>
       </c>
       <c r="D16" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="E16">
-        <v>0.174</v>
+        <v>0.281</v>
       </c>
       <c r="F16" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -994,13 +952,13 @@
         <v>21</v>
       </c>
       <c r="D17" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="E17">
-        <v>0.132</v>
+        <v>0.275</v>
       </c>
       <c r="F17" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1014,13 +972,13 @@
         <v>22</v>
       </c>
       <c r="D18" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="E18">
-        <v>0.13</v>
+        <v>0.268</v>
       </c>
       <c r="F18" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1034,13 +992,13 @@
         <v>23</v>
       </c>
       <c r="D19" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="E19">
-        <v>0.122</v>
+        <v>0.266</v>
       </c>
       <c r="F19" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1054,13 +1012,13 @@
         <v>24</v>
       </c>
       <c r="D20" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="E20">
-        <v>0.112</v>
+        <v>0.265</v>
       </c>
       <c r="F20" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1074,13 +1032,13 @@
         <v>25</v>
       </c>
       <c r="D21" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="E21">
-        <v>0.101</v>
+        <v>0.252</v>
       </c>
       <c r="F21" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -1094,13 +1052,13 @@
         <v>26</v>
       </c>
       <c r="D22" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="E22">
-        <v>0.099</v>
+        <v>0.245</v>
       </c>
       <c r="F22" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -1114,13 +1072,13 @@
         <v>27</v>
       </c>
       <c r="D23" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="E23">
-        <v>0.095</v>
+        <v>0.239</v>
       </c>
       <c r="F23" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -1134,13 +1092,13 @@
         <v>28</v>
       </c>
       <c r="D24" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E24">
-        <v>0.09</v>
+        <v>0.229</v>
       </c>
       <c r="F24" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -1154,13 +1112,13 @@
         <v>29</v>
       </c>
       <c r="D25" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="E25">
-        <v>0.08900000000000001</v>
+        <v>0.223</v>
       </c>
       <c r="F25" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -1174,13 +1132,13 @@
         <v>30</v>
       </c>
       <c r="D26" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="E26">
-        <v>0.083</v>
+        <v>0.21</v>
       </c>
       <c r="F26" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1194,13 +1152,13 @@
         <v>31</v>
       </c>
       <c r="D27" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="E27">
-        <v>0.08199999999999999</v>
+        <v>0.202</v>
       </c>
       <c r="F27" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1214,13 +1172,13 @@
         <v>32</v>
       </c>
       <c r="D28" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="E28">
-        <v>0.08</v>
+        <v>0.196</v>
       </c>
       <c r="F28" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1234,13 +1192,13 @@
         <v>33</v>
       </c>
       <c r="D29" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="E29">
-        <v>0.078</v>
+        <v>0.194</v>
       </c>
       <c r="F29" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1254,13 +1212,13 @@
         <v>34</v>
       </c>
       <c r="D30" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="E30">
-        <v>0.07200000000000001</v>
+        <v>0.192</v>
       </c>
       <c r="F30" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -1274,13 +1232,13 @@
         <v>35</v>
       </c>
       <c r="D31" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="E31">
-        <v>0.065</v>
+        <v>0.187</v>
       </c>
       <c r="F31" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -1294,13 +1252,13 @@
         <v>36</v>
       </c>
       <c r="D32" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="E32">
-        <v>0.065</v>
+        <v>0.187</v>
       </c>
       <c r="F32" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -1314,13 +1272,13 @@
         <v>37</v>
       </c>
       <c r="D33" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="E33">
-        <v>0.064</v>
+        <v>0.184</v>
       </c>
       <c r="F33" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -1334,13 +1292,13 @@
         <v>38</v>
       </c>
       <c r="D34" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="E34">
-        <v>0.052</v>
+        <v>0.169</v>
       </c>
       <c r="F34" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -1354,13 +1312,13 @@
         <v>39</v>
       </c>
       <c r="D35" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="E35">
-        <v>0.047</v>
+        <v>0.158</v>
       </c>
       <c r="F35" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -1374,153 +1332,13 @@
         <v>40</v>
       </c>
       <c r="D36" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="E36">
-        <v>0.044</v>
+        <v>0.149</v>
       </c>
       <c r="F36" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6">
-      <c r="A37" s="1">
-        <v>35</v>
-      </c>
-      <c r="B37" t="s">
-        <v>5</v>
-      </c>
-      <c r="C37" t="s">
-        <v>41</v>
-      </c>
-      <c r="D37" t="s">
-        <v>83</v>
-      </c>
-      <c r="E37">
-        <v>0.042</v>
-      </c>
-      <c r="F37" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6">
-      <c r="A38" s="1">
-        <v>36</v>
-      </c>
-      <c r="B38" t="s">
-        <v>5</v>
-      </c>
-      <c r="C38" t="s">
-        <v>42</v>
-      </c>
-      <c r="D38" t="s">
-        <v>84</v>
-      </c>
-      <c r="E38">
-        <v>0.038</v>
-      </c>
-      <c r="F38" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39" s="1">
-        <v>37</v>
-      </c>
-      <c r="B39" t="s">
-        <v>5</v>
-      </c>
-      <c r="C39" t="s">
-        <v>43</v>
-      </c>
-      <c r="D39" t="s">
-        <v>85</v>
-      </c>
-      <c r="E39">
-        <v>0.036</v>
-      </c>
-      <c r="F39" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="A40" s="1">
-        <v>38</v>
-      </c>
-      <c r="B40" t="s">
-        <v>5</v>
-      </c>
-      <c r="C40" t="s">
-        <v>44</v>
-      </c>
-      <c r="D40" t="s">
-        <v>86</v>
-      </c>
-      <c r="E40">
-        <v>0.033</v>
-      </c>
-      <c r="F40" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41" s="1">
-        <v>39</v>
-      </c>
-      <c r="B41" t="s">
-        <v>5</v>
-      </c>
-      <c r="C41" t="s">
-        <v>45</v>
-      </c>
-      <c r="D41" t="s">
-        <v>87</v>
-      </c>
-      <c r="E41">
-        <v>0.033</v>
-      </c>
-      <c r="F41" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6">
-      <c r="A42" s="1">
-        <v>40</v>
-      </c>
-      <c r="B42" t="s">
-        <v>5</v>
-      </c>
-      <c r="C42" t="s">
-        <v>46</v>
-      </c>
-      <c r="D42" t="s">
-        <v>88</v>
-      </c>
-      <c r="E42">
-        <v>0.032</v>
-      </c>
-      <c r="F42" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6">
-      <c r="A43" s="1">
-        <v>41</v>
-      </c>
-      <c r="B43" t="s">
-        <v>5</v>
-      </c>
-      <c r="C43" t="s">
-        <v>47</v>
-      </c>
-      <c r="D43" t="s">
-        <v>89</v>
-      </c>
-      <c r="E43">
-        <v>0.028</v>
-      </c>
-      <c r="F43" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>

</xml_diff>